<commit_message>
Update flowcharts and testing artifacts
</commit_message>
<xml_diff>
--- a/01_Planning/Release_Planning/QA_Workshop_Release_Planning.xlsx
+++ b/01_Planning/Release_Planning/QA_Workshop_Release_Planning.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shady gamal\OneDrive\Desktop\QA_Workshop\01_Planning\Release_Planning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{966E407C-D5A2-470A-9425-152A6D0B9B46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E035A2E-B0ED-42C0-B22C-C01B58EF55C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13152" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint_1" sheetId="1" r:id="rId1"/>
     <sheet name="📊 Dashboard" sheetId="2" r:id="rId2"/>
     <sheet name="Sprint_2" sheetId="3" r:id="rId3"/>
-    <sheet name="Sprint_3" sheetId="4" r:id="rId4"/>
+    <sheet name="Sprint_4" sheetId="5" r:id="rId4"/>
+    <sheet name="Sprint_3" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="52">
   <si>
     <t>📋  Sprint 1  —  QA Workshop Release Planning</t>
   </si>
@@ -192,6 +193,9 @@
   </si>
   <si>
     <t>📈  Sprint 3 — Team Hours Overview</t>
+  </si>
+  <si>
+    <t>📋  Sprint 4  —  QA Workshop Release Planning</t>
   </si>
 </sst>
 </file>
@@ -531,15 +535,15 @@
     <xf numFmtId="164" fontId="14" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1739,6 +1743,416 @@
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="1"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="1" i="0">
+                <a:solidFill>
+                  <a:srgbClr val="757575"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" b="1" i="0">
+                <a:solidFill>
+                  <a:srgbClr val="757575"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:rPr>
+              <a:t>Sprint </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="ar-EG" b="1" i="0">
+                <a:solidFill>
+                  <a:srgbClr val="757575"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:rPr>
+              <a:t>4</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" b="1" i="0">
+                <a:solidFill>
+                  <a:srgbClr val="757575"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:rPr>
+              <a:t>: Planned vs Actual Hours</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Planned Hours</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="3498DB"/>
+            </a:solidFill>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="1"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sprint_4!$A$61:$A$65</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>Omar Kandeel</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Abdelrahman Yasser</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Amr</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Amira</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Aya</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sprint_4!$B$61:$B$65</c:f>
+              <c:numCache>
+                <c:formatCode>0.0</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>14</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{6F2FDCE9-48DA-4B69-8628-5D25D57E5C99}">
+              <c14:invertSolidFillFmt>
+                <c14:spPr xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                  <a:ln cmpd="sng">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                  </a:ln>
+                </c14:spPr>
+              </c14:invertSolidFillFmt>
+            </c:ext>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-3B39-4FD1-9790-EE051662446B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Actual Hours</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="1A7A8A"/>
+            </a:solidFill>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="1"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sprint_4!$A$61:$A$65</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>Omar Kandeel</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Abdelrahman Yasser</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Amr</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Amira</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Aya</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sprint_4!$C$61:$C$65</c:f>
+              <c:numCache>
+                <c:formatCode>0.0</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>5.5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{6F2FDCE9-48DA-4B69-8628-5D25D57E5C99}">
+              <c14:invertSolidFillFmt>
+                <c14:spPr xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                  <a:ln cmpd="sng">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                  </a:ln>
+                </c14:spPr>
+              </c14:invertSolidFillFmt>
+            </c:ext>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-3B39-4FD1-9790-EE051662446B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:axId val="706879812"/>
+        <c:axId val="244469785"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="706879812"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="1" i="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" b="1" i="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:rPr>
+                  <a:t>Team Member</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="244469785"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="1"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="244469785"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="1" i="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" b="1" i="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:rPr>
+                  <a:t>Hours</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="0.0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="706879812"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr lvl="0">
+            <a:defRPr b="0">
+              <a:solidFill>
+                <a:srgbClr val="1A1A1A"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="zero"/>
+    <c:showDLblsOverMax val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="1"/>
   <c:style val="2"/>
   <c:chart>
     <c:title>
@@ -1756,7 +2170,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr b="1" i="0">
+              <a:rPr lang="en-US" b="1" i="0">
                 <a:solidFill>
                   <a:srgbClr val="757575"/>
                 </a:solidFill>
@@ -1978,7 +2392,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr b="1" i="0">
+                  <a:rPr lang="en-US" b="1" i="0">
                     <a:solidFill>
                       <a:srgbClr val="000000"/>
                     </a:solidFill>
@@ -2048,7 +2462,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr b="1" i="0">
+                  <a:rPr lang="en-US" b="1" i="0">
                     <a:solidFill>
                       <a:srgbClr val="000000"/>
                     </a:solidFill>
@@ -2228,6 +2642,44 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="8639175" cy="5038725"/>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D7A4FA8D-1156-4CB4-B419-BFAEA1A51B2E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
@@ -2480,7 +2932,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="29"/>
@@ -2491,7 +2943,7 @@
     </row>
     <row r="2" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="31" t="s">
+      <c r="A3" s="28" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="29"/>
@@ -2673,7 +3125,7 @@
     </row>
     <row r="13" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="31" t="s">
+      <c r="A14" s="28" t="s">
         <v>17</v>
       </c>
       <c r="B14" s="29"/>
@@ -2855,7 +3307,7 @@
     </row>
     <row r="24" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="25" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="31" t="s">
+      <c r="A25" s="28" t="s">
         <v>19</v>
       </c>
       <c r="B25" s="29"/>
@@ -3038,7 +3490,7 @@
     </row>
     <row r="35" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="36" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="31" t="s">
+      <c r="A36" s="28" t="s">
         <v>21</v>
       </c>
       <c r="B36" s="29"/>
@@ -3221,7 +3673,7 @@
     </row>
     <row r="46" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="47" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="31" t="s">
+      <c r="A47" s="28" t="s">
         <v>22</v>
       </c>
       <c r="B47" s="29"/>
@@ -3403,7 +3855,7 @@
     <row r="57" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="59" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="32" t="s">
+      <c r="A59" s="31" t="s">
         <v>23</v>
       </c>
       <c r="B59" s="29"/>
@@ -5803,7 +6255,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="32" t="s">
         <v>47</v>
       </c>
       <c r="B1" s="29"/>
@@ -5814,7 +6266,7 @@
     </row>
     <row r="2" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="31" t="s">
+      <c r="A3" s="28" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="29"/>
@@ -5955,7 +6407,7 @@
     </row>
     <row r="13" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="31" t="s">
+      <c r="A14" s="28" t="s">
         <v>17</v>
       </c>
       <c r="B14" s="29"/>
@@ -6096,7 +6548,7 @@
     </row>
     <row r="24" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="25" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="31" t="s">
+      <c r="A25" s="28" t="s">
         <v>19</v>
       </c>
       <c r="B25" s="29"/>
@@ -6237,7 +6689,7 @@
     </row>
     <row r="35" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="36" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="31" t="s">
+      <c r="A36" s="28" t="s">
         <v>21</v>
       </c>
       <c r="B36" s="29"/>
@@ -6378,7 +6830,7 @@
     </row>
     <row r="46" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="47" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="31" t="s">
+      <c r="A47" s="28" t="s">
         <v>22</v>
       </c>
       <c r="B47" s="29"/>
@@ -6520,7 +6972,7 @@
     <row r="57" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="59" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="32" t="s">
+      <c r="A59" s="31" t="s">
         <v>48</v>
       </c>
       <c r="B59" s="29"/>
@@ -7562,6 +8014,1891 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29A5D737-23EB-48AB-A2C2-E423AB00DE86}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F1000"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="40" customWidth="1"/>
+    <col min="7" max="26" width="8.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="32" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="30"/>
+    </row>
+    <row r="2" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="30"/>
+    </row>
+    <row r="4" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="10">
+        <v>5</v>
+      </c>
+      <c r="C5" s="10">
+        <v>5</v>
+      </c>
+      <c r="D5" s="10">
+        <f t="shared" ref="D5:D11" si="0">IF(AND(B5&lt;&gt;"",C5&lt;&gt;""),B5-C5,"")</f>
+        <v>0</v>
+      </c>
+      <c r="E5" s="15"/>
+      <c r="F5" s="5"/>
+    </row>
+    <row r="6" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="11">
+        <v>0</v>
+      </c>
+      <c r="C6" s="11">
+        <v>0</v>
+      </c>
+      <c r="D6" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E6" s="16"/>
+      <c r="F6" s="9"/>
+    </row>
+    <row r="7" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="10">
+        <v>0</v>
+      </c>
+      <c r="C7" s="10">
+        <v>0</v>
+      </c>
+      <c r="D7" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E7" s="15"/>
+      <c r="F7" s="5"/>
+    </row>
+    <row r="8" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="11">
+        <v>0</v>
+      </c>
+      <c r="C8" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="D8" s="11">
+        <f t="shared" si="0"/>
+        <v>-0.5</v>
+      </c>
+      <c r="E8" s="16"/>
+      <c r="F8" s="9"/>
+    </row>
+    <row r="9" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="10">
+        <v>1</v>
+      </c>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="E9" s="15"/>
+      <c r="F9" s="5"/>
+    </row>
+    <row r="10" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="11">
+        <v>1</v>
+      </c>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="E10" s="16"/>
+      <c r="F10" s="9"/>
+    </row>
+    <row r="11" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="10">
+        <v>4</v>
+      </c>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="E11" s="15"/>
+      <c r="F11" s="5"/>
+    </row>
+    <row r="12" spans="1:6" ht="27.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="13">
+        <f t="shared" ref="B12:D12" si="1">SUM(B5:B11)</f>
+        <v>11</v>
+      </c>
+      <c r="C12" s="13">
+        <f t="shared" si="1"/>
+        <v>5.5</v>
+      </c>
+      <c r="D12" s="13">
+        <f t="shared" si="1"/>
+        <v>-0.5</v>
+      </c>
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
+    </row>
+    <row r="13" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="14" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="29"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="30"/>
+    </row>
+    <row r="15" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16" s="10">
+        <v>5</v>
+      </c>
+      <c r="C16" s="10">
+        <v>5</v>
+      </c>
+      <c r="D16" s="10">
+        <f t="shared" ref="D16:D22" si="2">IF(AND(B16&lt;&gt;"",C16&lt;&gt;""),B16-C16,"")</f>
+        <v>0</v>
+      </c>
+      <c r="E16" s="15"/>
+      <c r="F16" s="5"/>
+    </row>
+    <row r="17" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17" s="11">
+        <v>0</v>
+      </c>
+      <c r="C17" s="11">
+        <v>0</v>
+      </c>
+      <c r="D17" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E17" s="16"/>
+      <c r="F17" s="9"/>
+    </row>
+    <row r="18" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18" s="10">
+        <v>0</v>
+      </c>
+      <c r="C18" s="10">
+        <v>0</v>
+      </c>
+      <c r="D18" s="10">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E18" s="15"/>
+      <c r="F18" s="5"/>
+    </row>
+    <row r="19" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" s="11">
+        <v>2</v>
+      </c>
+      <c r="C19" s="11">
+        <v>2</v>
+      </c>
+      <c r="D19" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E19" s="16"/>
+      <c r="F19" s="9"/>
+    </row>
+    <row r="20" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" s="10">
+        <v>3</v>
+      </c>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E20" s="15"/>
+      <c r="F20" s="5"/>
+    </row>
+    <row r="21" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" s="11">
+        <v>1</v>
+      </c>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E21" s="16"/>
+      <c r="F21" s="9"/>
+    </row>
+    <row r="22" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B22" s="10">
+        <v>3</v>
+      </c>
+      <c r="C22" s="10"/>
+      <c r="D22" s="10" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E22" s="15"/>
+      <c r="F22" s="5"/>
+    </row>
+    <row r="23" spans="1:6" ht="27.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B23" s="13">
+        <f t="shared" ref="B23:D23" si="3">SUM(B16:B22)</f>
+        <v>14</v>
+      </c>
+      <c r="C23" s="13">
+        <f t="shared" si="3"/>
+        <v>7</v>
+      </c>
+      <c r="D23" s="13">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="E23" s="14"/>
+      <c r="F23" s="14"/>
+    </row>
+    <row r="24" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="25" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="28" t="s">
+        <v>19</v>
+      </c>
+      <c r="B25" s="29"/>
+      <c r="C25" s="29"/>
+      <c r="D25" s="29"/>
+      <c r="E25" s="29"/>
+      <c r="F25" s="30"/>
+    </row>
+    <row r="26" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B27" s="10">
+        <v>5</v>
+      </c>
+      <c r="C27" s="10">
+        <v>5</v>
+      </c>
+      <c r="D27" s="10">
+        <f t="shared" ref="D27:D33" si="4">IF(AND(B27&lt;&gt;"",C27&lt;&gt;""),B27-C27,"")</f>
+        <v>0</v>
+      </c>
+      <c r="E27" s="15"/>
+      <c r="F27" s="5"/>
+    </row>
+    <row r="28" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B28" s="11">
+        <v>1</v>
+      </c>
+      <c r="C28" s="11">
+        <v>1</v>
+      </c>
+      <c r="D28" s="11">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="E28" s="16"/>
+      <c r="F28" s="9"/>
+    </row>
+    <row r="29" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B29" s="10">
+        <v>0</v>
+      </c>
+      <c r="C29" s="10">
+        <v>0</v>
+      </c>
+      <c r="D29" s="10">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="E29" s="15"/>
+      <c r="F29" s="5"/>
+    </row>
+    <row r="30" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B30" s="11">
+        <v>2</v>
+      </c>
+      <c r="C30" s="11">
+        <v>1</v>
+      </c>
+      <c r="D30" s="11">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="E30" s="16"/>
+      <c r="F30" s="9"/>
+    </row>
+    <row r="31" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B31" s="10">
+        <v>2</v>
+      </c>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="E31" s="15"/>
+      <c r="F31" s="5"/>
+    </row>
+    <row r="32" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B32" s="11">
+        <v>2</v>
+      </c>
+      <c r="C32" s="11"/>
+      <c r="D32" s="11" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="E32" s="16"/>
+      <c r="F32" s="9"/>
+    </row>
+    <row r="33" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B33" s="10">
+        <v>0</v>
+      </c>
+      <c r="C33" s="10"/>
+      <c r="D33" s="10" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="E33" s="15"/>
+      <c r="F33" s="5"/>
+    </row>
+    <row r="34" spans="1:6" ht="27.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B34" s="13">
+        <f t="shared" ref="B34:D34" si="5">SUM(B27:B33)</f>
+        <v>12</v>
+      </c>
+      <c r="C34" s="13">
+        <f t="shared" si="5"/>
+        <v>7</v>
+      </c>
+      <c r="D34" s="13">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+    </row>
+    <row r="35" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="36" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="B36" s="29"/>
+      <c r="C36" s="29"/>
+      <c r="D36" s="29"/>
+      <c r="E36" s="29"/>
+      <c r="F36" s="30"/>
+    </row>
+    <row r="37" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B38" s="10">
+        <v>5</v>
+      </c>
+      <c r="C38" s="10">
+        <v>5</v>
+      </c>
+      <c r="D38" s="10">
+        <f t="shared" ref="D38:D44" si="6">IF(AND(B38&lt;&gt;"",C38&lt;&gt;""),B38-C38,"")</f>
+        <v>0</v>
+      </c>
+      <c r="E38" s="15"/>
+      <c r="F38" s="5"/>
+    </row>
+    <row r="39" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B39" s="11">
+        <v>1</v>
+      </c>
+      <c r="C39" s="11">
+        <v>1</v>
+      </c>
+      <c r="D39" s="11">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="E39" s="16"/>
+      <c r="F39" s="9"/>
+    </row>
+    <row r="40" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B40" s="10">
+        <v>0</v>
+      </c>
+      <c r="C40" s="10">
+        <v>0</v>
+      </c>
+      <c r="D40" s="10">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="E40" s="15"/>
+      <c r="F40" s="5"/>
+    </row>
+    <row r="41" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B41" s="11">
+        <v>2</v>
+      </c>
+      <c r="C41" s="11">
+        <v>2</v>
+      </c>
+      <c r="D41" s="11">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="E41" s="16"/>
+      <c r="F41" s="9"/>
+    </row>
+    <row r="42" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B42" s="10">
+        <v>3</v>
+      </c>
+      <c r="C42" s="10"/>
+      <c r="D42" s="10" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="E42" s="15"/>
+      <c r="F42" s="5"/>
+    </row>
+    <row r="43" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B43" s="11">
+        <v>2</v>
+      </c>
+      <c r="C43" s="11"/>
+      <c r="D43" s="11" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="E43" s="16"/>
+      <c r="F43" s="9"/>
+    </row>
+    <row r="44" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B44" s="10">
+        <v>1</v>
+      </c>
+      <c r="C44" s="10"/>
+      <c r="D44" s="10" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="E44" s="15"/>
+      <c r="F44" s="5"/>
+    </row>
+    <row r="45" spans="1:6" ht="27.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B45" s="13">
+        <f t="shared" ref="B45:D45" si="7">SUM(B38:B44)</f>
+        <v>14</v>
+      </c>
+      <c r="C45" s="13">
+        <f t="shared" si="7"/>
+        <v>8</v>
+      </c>
+      <c r="D45" s="13">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="E45" s="14"/>
+      <c r="F45" s="14"/>
+    </row>
+    <row r="46" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="47" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="B47" s="29"/>
+      <c r="C47" s="29"/>
+      <c r="D47" s="29"/>
+      <c r="E47" s="29"/>
+      <c r="F47" s="30"/>
+    </row>
+    <row r="48" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B49" s="10">
+        <v>5</v>
+      </c>
+      <c r="C49" s="10">
+        <v>5</v>
+      </c>
+      <c r="D49" s="10">
+        <f t="shared" ref="D49:D55" si="8">IF(AND(B49&lt;&gt;"",C49&lt;&gt;""),B49-C49,"")</f>
+        <v>0</v>
+      </c>
+      <c r="E49" s="15"/>
+      <c r="F49" s="5"/>
+    </row>
+    <row r="50" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B50" s="11">
+        <v>1</v>
+      </c>
+      <c r="C50" s="11">
+        <v>1</v>
+      </c>
+      <c r="D50" s="11">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="E50" s="16"/>
+      <c r="F50" s="9"/>
+    </row>
+    <row r="51" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B51" s="10">
+        <v>0</v>
+      </c>
+      <c r="C51" s="10">
+        <v>0</v>
+      </c>
+      <c r="D51" s="10">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="E51" s="15"/>
+      <c r="F51" s="5"/>
+    </row>
+    <row r="52" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B52" s="11">
+        <v>2</v>
+      </c>
+      <c r="C52" s="11">
+        <v>2</v>
+      </c>
+      <c r="D52" s="11">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="E52" s="16"/>
+      <c r="F52" s="9"/>
+    </row>
+    <row r="53" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B53" s="10">
+        <v>3</v>
+      </c>
+      <c r="C53" s="10"/>
+      <c r="D53" s="10" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="E53" s="15"/>
+      <c r="F53" s="5"/>
+    </row>
+    <row r="54" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B54" s="11">
+        <v>2</v>
+      </c>
+      <c r="C54" s="11"/>
+      <c r="D54" s="11" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="E54" s="16"/>
+      <c r="F54" s="9"/>
+    </row>
+    <row r="55" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A55" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B55" s="10">
+        <v>1</v>
+      </c>
+      <c r="C55" s="10"/>
+      <c r="D55" s="10" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="E55" s="15"/>
+      <c r="F55" s="5"/>
+    </row>
+    <row r="56" spans="1:6" ht="27.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A56" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B56" s="13">
+        <f t="shared" ref="B56:D56" si="9">SUM(B49:B55)</f>
+        <v>14</v>
+      </c>
+      <c r="C56" s="13">
+        <f t="shared" si="9"/>
+        <v>8</v>
+      </c>
+      <c r="D56" s="13">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="E56" s="14"/>
+      <c r="F56" s="14"/>
+    </row>
+    <row r="57" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="58" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="59" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="31" t="s">
+        <v>50</v>
+      </c>
+      <c r="B59" s="29"/>
+      <c r="C59" s="29"/>
+      <c r="D59" s="29"/>
+      <c r="E59" s="29"/>
+      <c r="F59" s="30"/>
+    </row>
+    <row r="60" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B61" s="10">
+        <f t="shared" ref="B61:C61" si="10">B12</f>
+        <v>11</v>
+      </c>
+      <c r="C61" s="10">
+        <f t="shared" si="10"/>
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="B62" s="11">
+        <f t="shared" ref="B62:C62" si="11">B23</f>
+        <v>14</v>
+      </c>
+      <c r="C62" s="11">
+        <f t="shared" si="11"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B63" s="10">
+        <f t="shared" ref="B63:C63" si="12">B34</f>
+        <v>12</v>
+      </c>
+      <c r="C63" s="10">
+        <f t="shared" si="12"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B64" s="11">
+        <f t="shared" ref="B64:C64" si="13">B45</f>
+        <v>14</v>
+      </c>
+      <c r="C64" s="11">
+        <f t="shared" si="13"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B65" s="10">
+        <f t="shared" ref="B65:C65" si="14">B56</f>
+        <v>14</v>
+      </c>
+      <c r="C65" s="10">
+        <f t="shared" si="14"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="67" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="68" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="69" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="70" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="71" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="72" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="73" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="74" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="75" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="76" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="77" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="78" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="79" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="80" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="81" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="82" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="83" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="84" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="85" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="86" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="87" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="88" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="89" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="90" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="91" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="92" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="93" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="94" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="95" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="96" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="97" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="98" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="99" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="100" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="101" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="102" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="103" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="104" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="105" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="106" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="107" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="108" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="109" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="110" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="111" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="112" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="113" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="114" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="115" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="116" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="117" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="118" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="119" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="120" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="121" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="122" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="123" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="124" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="125" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="126" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="127" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="128" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="129" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="130" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="131" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="132" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="133" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="134" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="135" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="136" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="137" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="138" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="139" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="140" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="141" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="142" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="143" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="144" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="145" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="146" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="147" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="148" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="149" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="150" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="151" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="152" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="153" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="154" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="155" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="156" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="157" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="158" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="159" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="160" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="161" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="162" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="163" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="164" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="165" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="166" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="167" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="168" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="169" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="170" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="171" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="172" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="173" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="174" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="175" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="176" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="177" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="178" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="179" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="180" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="181" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="182" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="183" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="184" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="185" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="186" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="187" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="188" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="189" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="190" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="191" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="192" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="193" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="194" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="195" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="196" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="197" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="198" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="199" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="200" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="201" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="202" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="203" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="204" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="205" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="206" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="207" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="208" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="209" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="210" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="211" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="212" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="213" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="214" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="215" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="216" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="217" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="218" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="219" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="220" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="221" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="222" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="223" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="224" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="225" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="226" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="227" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="228" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="229" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="230" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="231" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="232" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="233" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="234" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="235" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="236" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="237" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="238" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="239" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="240" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="241" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="242" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="243" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="244" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="245" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="246" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="247" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="248" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="249" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="250" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="251" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="252" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="253" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="254" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="255" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="256" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="257" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="258" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="259" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="260" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="261" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="262" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="263" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="264" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="265" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="266" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="267" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="268" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="269" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="270" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="271" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="272" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="273" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="274" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="275" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="276" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="277" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="278" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="279" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="280" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="281" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="282" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="283" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="284" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="285" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="286" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="287" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="288" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="289" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="290" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="291" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="292" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="293" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="294" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="295" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="296" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="297" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="298" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="299" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="300" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="301" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="302" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="303" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="304" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="305" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="306" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="307" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="308" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="309" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="310" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="311" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="312" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="313" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="314" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="315" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="316" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="317" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="318" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="319" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="320" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="321" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="322" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="323" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="324" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="325" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="326" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="327" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="328" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="329" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="330" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="331" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="332" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="333" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="334" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="335" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="336" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="337" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="338" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="339" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="340" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="341" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="342" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="343" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="344" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="345" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="346" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="347" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="348" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="349" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="350" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="351" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="352" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="353" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="354" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="355" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="356" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="357" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="358" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="359" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="360" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="361" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="362" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="363" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="364" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="365" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="366" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="367" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="368" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="369" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="370" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="371" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="372" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="373" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="374" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="375" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="376" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="377" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="378" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="379" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="380" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="381" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="382" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="383" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="384" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="385" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="386" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="387" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="388" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="389" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="390" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="391" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="392" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="393" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="394" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="395" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="396" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="397" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="398" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="399" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="400" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="401" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="402" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="403" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="404" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="405" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="406" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="407" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="408" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="409" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="410" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="411" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="412" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="413" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="414" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="415" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="416" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="417" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="418" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="419" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="420" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="421" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="422" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="423" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="424" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="425" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="426" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="427" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="428" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="429" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="430" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="431" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="432" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="433" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="434" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="435" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="436" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="437" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="438" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="439" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="440" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="441" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="442" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="443" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="444" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="445" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="446" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="447" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="448" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="449" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="450" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="451" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="452" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="453" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="454" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="455" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="456" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="457" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="458" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="459" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="460" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="461" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="462" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="463" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="464" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="465" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="466" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="467" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="468" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="469" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="470" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="471" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="472" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="473" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="474" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="475" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="476" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="477" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="478" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="479" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="480" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="481" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="482" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="483" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="484" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="485" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="486" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="487" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="488" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="489" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="490" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="491" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="492" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="493" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="494" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="495" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="496" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="497" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="498" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="499" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="500" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="501" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="502" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="503" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="504" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="505" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="506" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="507" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="508" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="509" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="510" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="511" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="512" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="513" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="514" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="515" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="516" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="517" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="518" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="519" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="520" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="521" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="522" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="523" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="524" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="525" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="526" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="527" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="528" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="529" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="530" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="531" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="532" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="533" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="534" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="535" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="536" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="537" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="538" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="539" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="540" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="541" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="542" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="543" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="544" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="545" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="546" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="547" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="548" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="549" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="550" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="551" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="552" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="553" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="554" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="555" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="556" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="557" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="558" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="559" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="560" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="561" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="562" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="563" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="564" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="565" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="566" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="567" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="568" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="569" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="570" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="571" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="572" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="573" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="574" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="575" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="576" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="577" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="578" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="579" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="580" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="581" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="582" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="583" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="584" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="585" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="586" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="587" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="588" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="589" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="590" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="591" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="592" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="593" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="594" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="595" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="596" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="597" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="598" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="599" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="600" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="601" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="602" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="603" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="604" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="605" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="606" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="607" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="608" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="609" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="610" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="611" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="612" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="613" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="614" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="615" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="616" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="617" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="618" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="619" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="620" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="621" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="622" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="623" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="624" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="625" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="626" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="627" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="628" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="629" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="630" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="631" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="632" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="633" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="634" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="635" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="636" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="637" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="638" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="639" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="640" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="641" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="642" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="643" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="644" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="645" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="646" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="647" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="648" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="649" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="650" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="651" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="652" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="653" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="654" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="655" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="656" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="657" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="658" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="659" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="660" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="661" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="662" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="663" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="664" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="665" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="666" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="667" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="668" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="669" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="670" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="671" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="672" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="673" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="674" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="675" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="676" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="677" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="678" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="679" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="680" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="681" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="682" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="683" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="684" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="685" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="686" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="687" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="688" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="689" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="690" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="691" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="692" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="693" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="694" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="695" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="696" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="697" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="698" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="699" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="700" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="701" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="702" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="703" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="704" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="705" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="706" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="707" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="708" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="709" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="710" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="711" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="712" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="713" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="714" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="715" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="716" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="717" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="718" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="719" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="720" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="721" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="722" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="723" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="724" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="725" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="726" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="727" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="728" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="729" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="730" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="731" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="732" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="733" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="734" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="735" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="736" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="737" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="738" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="739" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="740" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="741" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="742" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="743" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="744" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="745" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="746" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="747" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="748" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="749" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="750" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="751" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="752" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="753" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="754" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="755" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="756" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="757" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="758" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="759" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="760" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="761" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="762" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="763" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="764" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="765" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="766" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="767" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="768" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="769" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="770" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="771" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="772" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="773" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="774" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="775" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="776" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="777" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="778" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="779" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="780" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="781" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="782" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="783" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="784" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="785" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="786" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="787" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="788" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="789" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="790" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="791" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="792" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="793" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="794" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="795" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="796" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="797" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="798" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="799" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="800" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="801" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="802" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="803" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="804" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="805" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="806" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="807" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="808" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="809" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="810" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="811" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="812" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="813" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="814" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="815" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="816" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="817" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="818" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="819" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="820" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="821" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="822" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="823" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="824" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="825" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="826" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="827" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="828" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="829" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="830" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="831" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="832" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="833" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="834" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="835" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="836" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="837" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="838" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="839" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="840" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="841" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="842" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="843" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="844" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="845" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="846" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="847" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="848" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="849" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="850" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="851" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="852" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="853" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="854" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="855" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="856" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="857" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="858" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="859" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="860" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="861" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="862" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="863" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="864" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="865" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="866" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="867" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="868" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="869" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="870" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="871" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="872" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="873" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="874" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="875" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="876" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="877" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="878" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="879" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="880" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="881" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="882" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="883" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="884" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="885" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="886" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="887" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="888" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="889" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="890" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="891" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="892" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="893" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="894" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="895" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="896" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="897" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="898" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="899" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="900" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="901" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="902" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="903" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="904" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="905" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="906" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="907" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="908" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="909" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="910" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="911" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="912" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="913" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="914" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="915" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="916" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="917" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="918" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="919" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="920" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="921" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="922" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="923" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="924" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="925" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="926" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="927" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="928" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="929" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="930" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="931" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="932" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="933" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="934" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="935" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="936" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="937" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="938" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="939" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="940" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="941" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="942" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="943" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="944" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="945" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="946" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="947" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="948" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="949" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="950" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="951" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="952" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="953" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="954" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="955" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="956" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="957" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="958" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="959" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="960" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="961" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="962" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="963" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="964" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="965" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="966" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="967" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="968" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="969" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="970" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="971" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="972" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="973" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="974" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="975" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="976" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="977" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="978" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="979" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="980" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="981" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="982" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="983" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="984" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="985" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="986" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="987" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="988" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="989" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="990" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="991" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="992" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="993" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="994" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="995" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="996" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="997" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="998" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="999" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="1000" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A59:F59"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A47:F47"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Status - Select task status" sqref="E5:E11 E16:E22 E27:E33 E38:E44 E49:E55" xr:uid="{693DB61B-E240-4124-A392-E4485A593AAC}">
+      <formula1>"✅ Done,🔄 In Progress,⏳ Not Started,⚠️ Blocked"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
+  <pageSetup fitToHeight="0" orientation="landscape"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -7578,7 +9915,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="32" t="s">
         <v>49</v>
       </c>
       <c r="B1" s="29"/>
@@ -7589,7 +9926,7 @@
     </row>
     <row r="2" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="31" t="s">
+      <c r="A3" s="28" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="29"/>
@@ -7730,7 +10067,7 @@
     </row>
     <row r="13" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="31" t="s">
+      <c r="A14" s="28" t="s">
         <v>17</v>
       </c>
       <c r="B14" s="29"/>
@@ -7871,7 +10208,7 @@
     </row>
     <row r="24" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="25" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="31" t="s">
+      <c r="A25" s="28" t="s">
         <v>19</v>
       </c>
       <c r="B25" s="29"/>
@@ -8012,7 +10349,7 @@
     </row>
     <row r="35" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="36" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="31" t="s">
+      <c r="A36" s="28" t="s">
         <v>21</v>
       </c>
       <c r="B36" s="29"/>
@@ -8153,7 +10490,7 @@
     </row>
     <row r="46" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="47" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="31" t="s">
+      <c r="A47" s="28" t="s">
         <v>22</v>
       </c>
       <c r="B47" s="29"/>
@@ -8295,7 +10632,7 @@
     <row r="57" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="59" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="32" t="s">
+      <c r="A59" s="31" t="s">
         <v>50</v>
       </c>
       <c r="B59" s="29"/>

</xml_diff>